<commit_message>
v3.1: gozlemci duyarliligi + 100 kontrol + K3 cikarimsal + PDF/Excel/full-repo
</commit_message>
<xml_diff>
--- a/09_teslim/sonuc-tablolari.xlsx
+++ b/09_teslim/sonuc-tablolari.xlsx
@@ -9206,13 +9206,17 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.0207</v>
-      </c>
-      <c r="B2" t="inlineStr"/>
+        <v>-0.0005</v>
+      </c>
+      <c r="B2" t="n">
+        <v>0.5258</v>
+      </c>
       <c r="C2" t="n">
-        <v>-0.1085</v>
-      </c>
-      <c r="D2" t="inlineStr"/>
+        <v>-0.1867</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.1889</v>
+      </c>
       <c r="E2" t="n">
         <v>5</v>
       </c>

</xml_diff>